<commit_message>
shablonlar: seed kodlari, bolim_kodi uchun izoh
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/employees-shablon.xlsx
+++ b/docs/templates/employees-shablon.xlsx
@@ -8,6 +8,23 @@
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="G2" authorId="0">
+      <text>
+        <r>
+          <t>avval /departments orqali yaratiladi</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -527,5 +544,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>